<commit_message>
feat: agentic-ai integration for tool selection, redis caching
</commit_message>
<xml_diff>
--- a/backend/data-filtering/database_export.xlsx
+++ b/backend/data-filtering/database_export.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\travel\backend\data-filtering\output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\travel\backend\data-filtering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF103AF-8853-4BBE-9F02-62821F44BB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73252C21-9631-4F45-9842-434613649F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2730,6 +2730,12 @@
       <c r="B83" t="s">
         <v>218</v>
       </c>
+      <c r="C83">
+        <v>19.218047741834301</v>
+      </c>
+      <c r="D83">
+        <v>73.086670500182706</v>
+      </c>
       <c r="E83" t="s">
         <v>147</v>
       </c>
@@ -2758,6 +2764,12 @@
       <c r="B85" t="s">
         <v>220</v>
       </c>
+      <c r="C85">
+        <v>19.130273573063398</v>
+      </c>
+      <c r="D85">
+        <v>72.821537864634394</v>
+      </c>
       <c r="E85" t="s">
         <v>138</v>
       </c>
@@ -2769,6 +2781,12 @@
       <c r="B86" t="s">
         <v>221</v>
       </c>
+      <c r="C86">
+        <v>19.128256625477601</v>
+      </c>
+      <c r="D86">
+        <v>72.8304696937535</v>
+      </c>
       <c r="E86" t="s">
         <v>138</v>
       </c>
@@ -2780,6 +2798,12 @@
       <c r="B87" t="s">
         <v>222</v>
       </c>
+      <c r="C87">
+        <v>19.126815547832798</v>
+      </c>
+      <c r="D87">
+        <v>72.837911919649002</v>
+      </c>
       <c r="E87" t="s">
         <v>138</v>
       </c>
@@ -2791,6 +2815,12 @@
       <c r="B88" t="s">
         <v>169</v>
       </c>
+      <c r="C88">
+        <v>19.120464334592501</v>
+      </c>
+      <c r="D88">
+        <v>72.848816658051703</v>
+      </c>
       <c r="E88" t="s">
         <v>138</v>
       </c>
@@ -2802,6 +2832,12 @@
       <c r="B89" t="s">
         <v>223</v>
       </c>
+      <c r="C89">
+        <v>19.115958088501401</v>
+      </c>
+      <c r="D89">
+        <v>72.856416863159097</v>
+      </c>
       <c r="E89" t="s">
         <v>138</v>
       </c>
@@ -2813,6 +2849,12 @@
       <c r="B90" t="s">
         <v>224</v>
       </c>
+      <c r="C90">
+        <v>19.111952294741599</v>
+      </c>
+      <c r="D90">
+        <v>72.868131203466604</v>
+      </c>
       <c r="E90" t="s">
         <v>138</v>
       </c>
@@ -2824,6 +2866,12 @@
       <c r="B91" t="s">
         <v>225</v>
       </c>
+      <c r="C91">
+        <v>19.110096732562301</v>
+      </c>
+      <c r="D91">
+        <v>72.874357897271395</v>
+      </c>
       <c r="E91" t="s">
         <v>138</v>
       </c>
@@ -2835,6 +2883,12 @@
       <c r="B92" t="s">
         <v>226</v>
       </c>
+      <c r="C92">
+        <v>19.108153982061999</v>
+      </c>
+      <c r="D92">
+        <v>72.879234088293998</v>
+      </c>
       <c r="E92" t="s">
         <v>138</v>
       </c>
@@ -2846,6 +2900,12 @@
       <c r="B93" t="s">
         <v>227</v>
       </c>
+      <c r="C93">
+        <v>19.103457457029702</v>
+      </c>
+      <c r="D93">
+        <v>72.888195725034905</v>
+      </c>
       <c r="E93" t="s">
         <v>138</v>
       </c>
@@ -2857,6 +2917,12 @@
       <c r="B94" t="s">
         <v>228</v>
       </c>
+      <c r="C94">
+        <v>19.096391816437599</v>
+      </c>
+      <c r="D94">
+        <v>72.895012171401405</v>
+      </c>
       <c r="E94" t="s">
         <v>138</v>
       </c>
@@ -2868,6 +2934,12 @@
       <c r="B95" t="s">
         <v>229</v>
       </c>
+      <c r="C95">
+        <v>19.0924169711597</v>
+      </c>
+      <c r="D95">
+        <v>72.902198182771698</v>
+      </c>
       <c r="E95" t="s">
         <v>138</v>
       </c>
@@ -2879,6 +2951,12 @@
       <c r="B96" t="s">
         <v>230</v>
       </c>
+      <c r="C96">
+        <v>19.087006098328398</v>
+      </c>
+      <c r="D96">
+        <v>72.908102062517898</v>
+      </c>
       <c r="E96" t="s">
         <v>138</v>
       </c>
@@ -2890,6 +2968,12 @@
       <c r="B97" t="s">
         <v>232</v>
       </c>
+      <c r="C97">
+        <v>19.125834143793199</v>
+      </c>
+      <c r="D97">
+        <v>72.873649450803896</v>
+      </c>
       <c r="E97" t="s">
         <v>138</v>
       </c>
@@ -2901,6 +2985,12 @@
       <c r="B98" t="s">
         <v>234</v>
       </c>
+      <c r="C98">
+        <v>19.131074143921701</v>
+      </c>
+      <c r="D98">
+        <v>72.884530524701603</v>
+      </c>
       <c r="E98" t="s">
         <v>138</v>
       </c>
@@ -2912,6 +3002,12 @@
       <c r="B99" t="s">
         <v>236</v>
       </c>
+      <c r="C99">
+        <v>19.117321331284</v>
+      </c>
+      <c r="D99">
+        <v>72.873858114032302</v>
+      </c>
       <c r="E99" t="s">
         <v>138</v>
       </c>
@@ -2923,6 +3019,12 @@
       <c r="B100" t="s">
         <v>226</v>
       </c>
+      <c r="C100">
+        <v>19.108236412342901</v>
+      </c>
+      <c r="D100">
+        <v>72.878664438111997</v>
+      </c>
       <c r="E100" t="s">
         <v>138</v>
       </c>
@@ -2934,6 +3036,12 @@
       <c r="B101" t="s">
         <v>239</v>
       </c>
+      <c r="C101">
+        <v>19.101995738104801</v>
+      </c>
+      <c r="D101">
+        <v>72.874427543867498</v>
+      </c>
       <c r="E101" t="s">
         <v>138</v>
       </c>
@@ -2945,6 +3053,12 @@
       <c r="B102" t="s">
         <v>241</v>
       </c>
+      <c r="C102">
+        <v>19.102156354286201</v>
+      </c>
+      <c r="D102">
+        <v>72.864775209224703</v>
+      </c>
       <c r="E102" t="s">
         <v>138</v>
       </c>
@@ -2956,6 +3070,12 @@
       <c r="B103" t="s">
         <v>243</v>
       </c>
+      <c r="C103">
+        <v>19.093919123267799</v>
+      </c>
+      <c r="D103">
+        <v>72.853459773607597</v>
+      </c>
       <c r="E103" t="s">
         <v>138</v>
       </c>
@@ -2967,6 +3087,12 @@
       <c r="B104" t="s">
         <v>245</v>
       </c>
+      <c r="C104">
+        <v>19.079021779316601</v>
+      </c>
+      <c r="D104">
+        <v>72.846878959936802</v>
+      </c>
       <c r="E104" t="s">
         <v>138</v>
       </c>
@@ -2978,6 +3104,12 @@
       <c r="B105" t="s">
         <v>247</v>
       </c>
+      <c r="C105">
+        <v>19.0699753347259</v>
+      </c>
+      <c r="D105">
+        <v>72.849433646359003</v>
+      </c>
       <c r="E105" t="s">
         <v>138</v>
       </c>
@@ -2989,6 +3121,12 @@
       <c r="B106" t="s">
         <v>249</v>
       </c>
+      <c r="C106">
+        <v>19.0604133069135</v>
+      </c>
+      <c r="D106">
+        <v>72.854924836254995</v>
+      </c>
       <c r="E106" t="s">
         <v>138</v>
       </c>
@@ -3000,6 +3138,12 @@
       <c r="B107" t="s">
         <v>251</v>
       </c>
+      <c r="C107">
+        <v>19.046276956102101</v>
+      </c>
+      <c r="D107">
+        <v>72.849935167801902</v>
+      </c>
       <c r="E107" t="s">
         <v>138</v>
       </c>
@@ -3011,6 +3155,12 @@
       <c r="B108" t="s">
         <v>253</v>
       </c>
+      <c r="C108">
+        <v>19.038298037905601</v>
+      </c>
+      <c r="D108">
+        <v>72.842127273159406</v>
+      </c>
       <c r="E108" t="s">
         <v>138</v>
       </c>
@@ -3022,6 +3172,12 @@
       <c r="B109" t="s">
         <v>255</v>
       </c>
+      <c r="C109">
+        <v>19.0228695408363</v>
+      </c>
+      <c r="D109">
+        <v>72.838566304946099</v>
+      </c>
       <c r="E109" t="s">
         <v>138</v>
       </c>
@@ -3033,6 +3189,12 @@
       <c r="B110" t="s">
         <v>257</v>
       </c>
+      <c r="C110">
+        <v>19.0172122834934</v>
+      </c>
+      <c r="D110">
+        <v>72.8303269127058</v>
+      </c>
       <c r="E110" t="s">
         <v>138</v>
       </c>
@@ -3044,6 +3206,12 @@
       <c r="B111" t="s">
         <v>259</v>
       </c>
+      <c r="C111">
+        <v>19.008692083428901</v>
+      </c>
+      <c r="D111">
+        <v>72.819399387525493</v>
+      </c>
       <c r="E111" t="s">
         <v>138</v>
       </c>
@@ -3055,6 +3223,12 @@
       <c r="B112" t="s">
         <v>261</v>
       </c>
+      <c r="C112">
+        <v>18.997148548784299</v>
+      </c>
+      <c r="D112">
+        <v>72.818174731505096</v>
+      </c>
       <c r="E112" t="s">
         <v>138</v>
       </c>
@@ -3066,6 +3240,12 @@
       <c r="B113" t="s">
         <v>263</v>
       </c>
+      <c r="C113">
+        <v>18.9903123764553</v>
+      </c>
+      <c r="D113">
+        <v>72.821770578483907</v>
+      </c>
       <c r="E113" t="s">
         <v>138</v>
       </c>
@@ -3077,6 +3257,12 @@
       <c r="B114" t="s">
         <v>265</v>
       </c>
+      <c r="C114">
+        <v>18.979455838643201</v>
+      </c>
+      <c r="D114">
+        <v>72.825329863269999</v>
+      </c>
       <c r="E114" t="s">
         <v>138</v>
       </c>
@@ -3088,6 +3274,12 @@
       <c r="B115" t="s">
         <v>266</v>
       </c>
+      <c r="C115">
+        <v>18.970600447171101</v>
+      </c>
+      <c r="D115">
+        <v>72.821381960734897</v>
+      </c>
       <c r="E115" t="s">
         <v>147</v>
       </c>
@@ -3099,6 +3291,12 @@
       <c r="B116" t="s">
         <v>268</v>
       </c>
+      <c r="C116">
+        <v>18.9705877849341</v>
+      </c>
+      <c r="D116">
+        <v>72.821393535316503</v>
+      </c>
       <c r="E116" t="s">
         <v>138</v>
       </c>
@@ -3110,6 +3308,12 @@
       <c r="B117" t="s">
         <v>270</v>
       </c>
+      <c r="C117">
+        <v>18.962967902985799</v>
+      </c>
+      <c r="D117">
+        <v>72.8181452721483</v>
+      </c>
       <c r="E117" t="s">
         <v>138</v>
       </c>
@@ -3121,6 +3325,12 @@
       <c r="B118" t="s">
         <v>272</v>
       </c>
+      <c r="C118">
+        <v>18.951912875698</v>
+      </c>
+      <c r="D118">
+        <v>72.822581551694299</v>
+      </c>
       <c r="E118" t="s">
         <v>138</v>
       </c>
@@ -3132,6 +3342,12 @@
       <c r="B119" t="s">
         <v>274</v>
       </c>
+      <c r="C119">
+        <v>18.9468802723284</v>
+      </c>
+      <c r="D119">
+        <v>72.826891711860895</v>
+      </c>
       <c r="E119" t="s">
         <v>138</v>
       </c>
@@ -3143,6 +3359,12 @@
       <c r="B120" t="s">
         <v>276</v>
       </c>
+      <c r="C120">
+        <v>18.940081054142802</v>
+      </c>
+      <c r="D120">
+        <v>72.8341244941968</v>
+      </c>
       <c r="E120" t="s">
         <v>138</v>
       </c>
@@ -3154,6 +3376,12 @@
       <c r="B121" t="s">
         <v>278</v>
       </c>
+      <c r="C121">
+        <v>18.9345762661316</v>
+      </c>
+      <c r="D121">
+        <v>72.832768697636297</v>
+      </c>
       <c r="E121" t="s">
         <v>138</v>
       </c>
@@ -3165,6 +3393,12 @@
       <c r="B122" t="s">
         <v>280</v>
       </c>
+      <c r="C122">
+        <v>18.930653325697499</v>
+      </c>
+      <c r="D122">
+        <v>72.826106667428405</v>
+      </c>
       <c r="E122" t="s">
         <v>138</v>
       </c>
@@ -3176,6 +3410,12 @@
       <c r="B123" t="s">
         <v>282</v>
       </c>
+      <c r="C123">
+        <v>18.9247406936618</v>
+      </c>
+      <c r="D123">
+        <v>72.825630212621604</v>
+      </c>
       <c r="E123" t="s">
         <v>138</v>
       </c>
@@ -3187,6 +3427,12 @@
       <c r="B124" t="s">
         <v>284</v>
       </c>
+      <c r="C124">
+        <v>18.912946686309098</v>
+      </c>
+      <c r="D124">
+        <v>72.820175202301996</v>
+      </c>
       <c r="E124" t="s">
         <v>138</v>
       </c>
@@ -3572,6 +3818,12 @@
       <c r="B147" t="s">
         <v>303</v>
       </c>
+      <c r="C147">
+        <v>19.211218716181602</v>
+      </c>
+      <c r="D147">
+        <v>73.077455860930897</v>
+      </c>
       <c r="E147" t="s">
         <v>147</v>
       </c>
@@ -3583,6 +3835,12 @@
       <c r="B148" t="s">
         <v>304</v>
       </c>
+      <c r="C148">
+        <v>19.235790061446298</v>
+      </c>
+      <c r="D148">
+        <v>73.131999404666502</v>
+      </c>
       <c r="E148" t="s">
         <v>147</v>
       </c>
@@ -3594,6 +3852,12 @@
       <c r="B149" t="s">
         <v>305</v>
       </c>
+      <c r="C149">
+        <v>19.228676550636902</v>
+      </c>
+      <c r="D149">
+        <v>73.148812891128998</v>
+      </c>
       <c r="E149" t="s">
         <v>147</v>
       </c>
@@ -3605,6 +3869,12 @@
       <c r="B150" t="s">
         <v>306</v>
       </c>
+      <c r="C150">
+        <v>19.217729688845001</v>
+      </c>
+      <c r="D150">
+        <v>73.163884457521107</v>
+      </c>
       <c r="E150" t="s">
         <v>147</v>
       </c>
@@ -3616,6 +3886,12 @@
       <c r="B151" t="s">
         <v>307</v>
       </c>
+      <c r="C151">
+        <v>19.209986451030598</v>
+      </c>
+      <c r="D151">
+        <v>73.184813019961197</v>
+      </c>
       <c r="E151" t="s">
         <v>147</v>
       </c>
@@ -3627,6 +3903,12 @@
       <c r="B152" t="s">
         <v>308</v>
       </c>
+      <c r="C152">
+        <v>19.166854940467701</v>
+      </c>
+      <c r="D152">
+        <v>73.238694145572893</v>
+      </c>
       <c r="E152" t="s">
         <v>147</v>
       </c>
@@ -3638,6 +3920,12 @@
       <c r="B153" t="s">
         <v>309</v>
       </c>
+      <c r="C153">
+        <v>19.094367640780799</v>
+      </c>
+      <c r="D153">
+        <v>73.300915701928403</v>
+      </c>
       <c r="E153" t="s">
         <v>147</v>
       </c>
@@ -3649,6 +3937,12 @@
       <c r="B154" t="s">
         <v>310</v>
       </c>
+      <c r="C154">
+        <v>19.063491239323501</v>
+      </c>
+      <c r="D154">
+        <v>73.317887513649694</v>
+      </c>
       <c r="E154" t="s">
         <v>147</v>
       </c>
@@ -3660,6 +3954,12 @@
       <c r="B155" t="s">
         <v>311</v>
       </c>
+      <c r="C155">
+        <v>19.026908648206099</v>
+      </c>
+      <c r="D155">
+        <v>73.318648079853105</v>
+      </c>
       <c r="E155" t="s">
         <v>147</v>
       </c>
@@ -3671,6 +3971,12 @@
       <c r="B156" t="s">
         <v>312</v>
       </c>
+      <c r="C156">
+        <v>18.971485875154801</v>
+      </c>
+      <c r="D156">
+        <v>73.331460734429498</v>
+      </c>
       <c r="E156" t="s">
         <v>147</v>
       </c>
@@ -3682,6 +3988,12 @@
       <c r="B157" t="s">
         <v>313</v>
       </c>
+      <c r="C157">
+        <v>18.910008639915699</v>
+      </c>
+      <c r="D157">
+        <v>73.320884491071794</v>
+      </c>
       <c r="E157" t="s">
         <v>147</v>
       </c>
@@ -3693,6 +4005,12 @@
       <c r="B158" t="s">
         <v>314</v>
       </c>
+      <c r="C158">
+        <v>18.8839997509426</v>
+      </c>
+      <c r="D158">
+        <v>73.320971526778905</v>
+      </c>
       <c r="E158" t="s">
         <v>147</v>
       </c>
@@ -3704,6 +4022,12 @@
       <c r="B159" t="s">
         <v>315</v>
       </c>
+      <c r="C159">
+        <v>18.845395373982001</v>
+      </c>
+      <c r="D159">
+        <v>73.318883584972994</v>
+      </c>
       <c r="E159" t="s">
         <v>147</v>
       </c>
@@ -3715,6 +4039,12 @@
       <c r="B160" t="s">
         <v>316</v>
       </c>
+      <c r="C160">
+        <v>18.833510918036399</v>
+      </c>
+      <c r="D160">
+        <v>73.320255172554695</v>
+      </c>
       <c r="E160" t="s">
         <v>147</v>
       </c>
@@ -3726,6 +4056,12 @@
       <c r="B161" t="s">
         <v>317</v>
       </c>
+      <c r="C161">
+        <v>18.809082112637601</v>
+      </c>
+      <c r="D161">
+        <v>73.335411319515401</v>
+      </c>
       <c r="E161" t="s">
         <v>147</v>
       </c>
@@ -3737,6 +4073,12 @@
       <c r="B162" t="s">
         <v>318</v>
       </c>
+      <c r="C162">
+        <v>18.788447404389</v>
+      </c>
+      <c r="D162">
+        <v>73.3459968666848</v>
+      </c>
       <c r="E162" t="s">
         <v>147</v>
       </c>
@@ -3748,6 +4090,12 @@
       <c r="B163" t="s">
         <v>319</v>
       </c>
+      <c r="C163">
+        <v>19.2442256159054</v>
+      </c>
+      <c r="D163">
+        <v>73.158255662646496</v>
+      </c>
       <c r="E163" t="s">
         <v>147</v>
       </c>
@@ -3759,6 +4107,12 @@
       <c r="B164" t="s">
         <v>320</v>
       </c>
+      <c r="C164">
+        <v>19.2683753970291</v>
+      </c>
+      <c r="D164">
+        <v>73.172056821648894</v>
+      </c>
       <c r="E164" t="s">
         <v>147</v>
       </c>
@@ -3770,6 +4124,12 @@
       <c r="B165" t="s">
         <v>321</v>
       </c>
+      <c r="C165">
+        <v>19.296323458805801</v>
+      </c>
+      <c r="D165">
+        <v>73.203204606576193</v>
+      </c>
       <c r="E165" t="s">
         <v>147</v>
       </c>
@@ -3781,6 +4141,12 @@
       <c r="B166" t="s">
         <v>322</v>
       </c>
+      <c r="C166">
+        <v>19.356615317294299</v>
+      </c>
+      <c r="D166">
+        <v>73.218846784330694</v>
+      </c>
       <c r="E166" t="s">
         <v>147</v>
       </c>
@@ -3792,6 +4158,12 @@
       <c r="B167" t="s">
         <v>323</v>
       </c>
+      <c r="C167">
+        <v>19.406564751639699</v>
+      </c>
+      <c r="D167">
+        <v>73.2673171150917</v>
+      </c>
       <c r="E167" t="s">
         <v>147</v>
       </c>
@@ -3803,6 +4175,12 @@
       <c r="B168" t="s">
         <v>324</v>
       </c>
+      <c r="C168">
+        <v>19.439507214603999</v>
+      </c>
+      <c r="D168">
+        <v>73.307871674232899</v>
+      </c>
       <c r="E168" t="s">
         <v>147</v>
       </c>
@@ -3814,6 +4192,12 @@
       <c r="B169" t="s">
         <v>325</v>
       </c>
+      <c r="C169">
+        <v>19.5206232179126</v>
+      </c>
+      <c r="D169">
+        <v>73.320594309677006</v>
+      </c>
       <c r="E169" t="s">
         <v>147</v>
       </c>
@@ -3825,6 +4209,12 @@
       <c r="B170" t="s">
         <v>326</v>
       </c>
+      <c r="C170">
+        <v>19.550188836253</v>
+      </c>
+      <c r="D170">
+        <v>73.351984343602595</v>
+      </c>
       <c r="E170" t="s">
         <v>147</v>
       </c>
@@ -3836,6 +4226,12 @@
       <c r="B171" t="s">
         <v>327</v>
       </c>
+      <c r="C171">
+        <v>19.5802433405823</v>
+      </c>
+      <c r="D171">
+        <v>73.3937655673314</v>
+      </c>
       <c r="E171" t="s">
         <v>147</v>
       </c>
@@ -3847,6 +4243,12 @@
       <c r="B172" t="s">
         <v>328</v>
       </c>
+      <c r="C172">
+        <v>19.628297953569199</v>
+      </c>
+      <c r="D172">
+        <v>73.422971124314401</v>
+      </c>
       <c r="E172" t="s">
         <v>147</v>
       </c>
@@ -3857,6 +4259,12 @@
       </c>
       <c r="B173" t="s">
         <v>329</v>
+      </c>
+      <c r="C173">
+        <v>19.6481503893229</v>
+      </c>
+      <c r="D173">
+        <v>73.4729406011718</v>
       </c>
       <c r="E173" t="s">
         <v>147</v>

</xml_diff>